<commit_message>
added DAP Logic for CSM
</commit_message>
<xml_diff>
--- a/CSM/CSM Verb and noun list.xlsx
+++ b/CSM/CSM Verb and noun list.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\del13\nassp-checklist-annotator\CSM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C284C39-955A-4965-A772-30A11BE62D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C26778-1970-470D-AF33-391302D52467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20388" yWindow="0" windowWidth="20664" windowHeight="16560" xr2:uid="{424832EF-970A-4448-8501-E17666F9A823}"/>
+    <workbookView xWindow="40764" yWindow="0" windowWidth="20616" windowHeight="16560" activeTab="4" xr2:uid="{424832EF-970A-4448-8501-E17666F9A823}"/>
   </bookViews>
   <sheets>
     <sheet name="Verb" sheetId="1" r:id="rId1"/>
     <sheet name="Noun" sheetId="2" r:id="rId2"/>
     <sheet name="Program" sheetId="3" r:id="rId3"/>
+    <sheet name="R1 DAP" sheetId="4" r:id="rId4"/>
+    <sheet name="R2 DAP" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -75,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="388">
   <si>
     <t>Display Fixed Memory</t>
   </si>
@@ -1149,6 +1151,96 @@
   </si>
   <si>
     <t>Display Decimal</t>
+  </si>
+  <si>
+    <t>CFG=1=CSMONLY</t>
+  </si>
+  <si>
+    <t>CFG=2=CSM&amp;LM</t>
+  </si>
+  <si>
+    <t>CFG=3=CSM&amp;SIVB</t>
+  </si>
+  <si>
+    <t>A/C=1=Use</t>
+  </si>
+  <si>
+    <t>CFG=0=NODAP</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>A/C=0=Fail</t>
+  </si>
+  <si>
+    <t>B/D=0=Fail</t>
+  </si>
+  <si>
+    <t>B/D=1=Use</t>
+  </si>
+  <si>
+    <t>DB=1=5.0°</t>
+  </si>
+  <si>
+    <t>DB=0=0.5°</t>
+  </si>
+  <si>
+    <t>RATE=0=0.05°/sec</t>
+  </si>
+  <si>
+    <t>RATE=1=0.2°/sec</t>
+  </si>
+  <si>
+    <t>RATE=2=0.5°/sec</t>
+  </si>
+  <si>
+    <t>RATE=3=2.0°/sec</t>
+  </si>
+  <si>
+    <t>ROLLQD=0=B/D</t>
+  </si>
+  <si>
+    <t>QDA=1=Use</t>
+  </si>
+  <si>
+    <t>QBD=1=Use</t>
+  </si>
+  <si>
+    <t>QDC=0=Fail</t>
+  </si>
+  <si>
+    <t>QDC=1=Use</t>
+  </si>
+  <si>
+    <t>QDD=0=Fail</t>
+  </si>
+  <si>
+    <t>QDD=1=Use</t>
+  </si>
+  <si>
+    <t>QDB=0=Fail</t>
+  </si>
+  <si>
+    <t>QDA=0=Fail</t>
+  </si>
+  <si>
+    <t>ROLLQD=1=A/C</t>
+  </si>
+  <si>
+    <t>CFG=6=CSM&amp;LMASC</t>
   </si>
 </sst>
 </file>
@@ -3624,4 +3716,181 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9961D1FC-420C-4232-8808-00D6568A027E}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>363</v>
+      </c>
+      <c r="C1" t="s">
+        <v>364</v>
+      </c>
+      <c r="D1" t="s">
+        <v>365</v>
+      </c>
+      <c r="E1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F1" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C3" t="s">
+        <v>361</v>
+      </c>
+      <c r="D3" t="s">
+        <v>370</v>
+      </c>
+      <c r="E3" t="s">
+        <v>371</v>
+      </c>
+      <c r="F3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>359</v>
+      </c>
+      <c r="F4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>360</v>
+      </c>
+      <c r="F5" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>387</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59C3EEC8-AB12-4CC1-8A27-0FC57B0E86B5}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>363</v>
+      </c>
+      <c r="C1" t="s">
+        <v>364</v>
+      </c>
+      <c r="D1" t="s">
+        <v>365</v>
+      </c>
+      <c r="E1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F1" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D2" t="s">
+        <v>384</v>
+      </c>
+      <c r="E2" t="s">
+        <v>380</v>
+      </c>
+      <c r="F2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C3" t="s">
+        <v>378</v>
+      </c>
+      <c r="D3" t="s">
+        <v>379</v>
+      </c>
+      <c r="E3" t="s">
+        <v>381</v>
+      </c>
+      <c r="F3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
found the delta symbol does not work, replaced with lowercase d
</commit_message>
<xml_diff>
--- a/CSM/CSM Verb and noun list.xlsx
+++ b/CSM/CSM Verb and noun list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\del13\nassp-checklist-annotator\CSM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C26778-1970-470D-AF33-391302D52467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A06BFA-0BBE-4C49-91F3-04D871F50276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40764" yWindow="0" windowWidth="20616" windowHeight="16560" activeTab="4" xr2:uid="{424832EF-970A-4448-8501-E17666F9A823}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20676" windowHeight="16560" activeTab="1" xr2:uid="{424832EF-970A-4448-8501-E17666F9A823}"/>
   </bookViews>
   <sheets>
     <sheet name="Verb" sheetId="1" r:id="rId1"/>
@@ -652,9 +652,6 @@
     <t>39</t>
   </si>
   <si>
-    <t>Δ Time of Transfer</t>
-  </si>
-  <si>
     <t>min-sec .1 FPS .1 FPS</t>
   </si>
   <si>
@@ -856,9 +853,6 @@
     <t>Optics Calibration / Cislunar Midcourse Nav. Meas.</t>
   </si>
   <si>
-    <t>External ΔV</t>
-  </si>
-  <si>
     <t>CSI Prethrust</t>
   </si>
   <si>
@@ -892,9 +886,6 @@
     <t>Entry Preparation</t>
   </si>
   <si>
-    <t>Target ΔV</t>
-  </si>
-  <si>
     <t>Program</t>
   </si>
   <si>
@@ -973,15 +964,9 @@
     <t>R1=Add +1 of error, R2=B BANK + SUPERBANK, R3=No of SELF TEST errors</t>
   </si>
   <si>
-    <t>R1=TF GETI/TFC, R2=VG, R3=ΔV (Accumulated)</t>
-  </si>
-  <si>
     <t>R1=Target Azimuth, R2=Target Elevation, R3=Target Ident</t>
   </si>
   <si>
-    <t>R1=Apogee Alt (HA), R2=Perigee Alt (HP), R3=ΔV (Required)</t>
-  </si>
-  <si>
     <t>R1=Lat (+ North), R2=Long (+ East), R3=Alt</t>
   </si>
   <si>
@@ -991,9 +976,6 @@
     <t>R1=Marks, R2 =TF GETI of next burn, R3=MGA</t>
   </si>
   <si>
-    <t>R1=ΔR, R2=ΔV, R3=SOURCE CODE (1 optics,2 VHF)</t>
-  </si>
-  <si>
     <t>R1=RANGE, R2=RANGE RATE, R3=PHI (lcl horiz)</t>
   </si>
   <si>
@@ -1120,36 +1102,6 @@
     <t>Landmark, R1=Lat (+ North), R2=Long/2 (+ East), R3=Alt</t>
   </si>
   <si>
-    <t>R1=ΔR (miss distance, R2=PERIGEE (HP), R3=TFF</t>
-  </si>
-  <si>
-    <t>ΔR offset (SOR) (+ indicates behind target)</t>
-  </si>
-  <si>
-    <t>R1=HP alt (post TPI)(SOR for P38), R2=ΔV (TPI)(SOR for P38), R3=ΔV (TPF)(SOR FINAL for P38)</t>
-  </si>
-  <si>
-    <t>R1=ΔV LOS 1, R2=ΔV LOS 2, R3=ΔV LOS 3</t>
-  </si>
-  <si>
-    <t>R1=Δ ang, R2=Δ alt, Search option</t>
-  </si>
-  <si>
-    <t>R1=ΔH (CDH), R2=ΔT, R3=ΔT</t>
-  </si>
-  <si>
-    <t>ΔVX,Y,Z (lcl vert)</t>
-  </si>
-  <si>
-    <t>ΔVX,Y,Z (LV) CDH</t>
-  </si>
-  <si>
-    <t>ΔVX,Y,Z (Body Control Axis)</t>
-  </si>
-  <si>
-    <t>ΔVX,Y,Z (Other Vehicle)</t>
-  </si>
-  <si>
     <t>Display Decimal</t>
   </si>
   <si>
@@ -1241,6 +1193,54 @@
   </si>
   <si>
     <t>CFG=6=CSM&amp;LMASC</t>
+  </si>
+  <si>
+    <t>d Time of Transfer</t>
+  </si>
+  <si>
+    <t>R1=TF GETI/TFC, R2=VG, R3=dV (Accumulated)</t>
+  </si>
+  <si>
+    <t>R1=Apogee Alt (HA), R2=Perigee Alt (HP), R3=dV (Required)</t>
+  </si>
+  <si>
+    <t>R1=dR, R2=dV, R3=SOURCE CODE (1 optics,2 VHF)</t>
+  </si>
+  <si>
+    <t>R1=dR (miss distance, R2=PERIGEE (HP), R3=TFF</t>
+  </si>
+  <si>
+    <t>dR offset (SOR) (+ indicates behind target)</t>
+  </si>
+  <si>
+    <t>R1=HP alt (post TPI)(SOR for P38), R2=dV (TPI)(SOR for P38), R3=dV (TPF)(SOR FINAL for P38)</t>
+  </si>
+  <si>
+    <t>R1=dV LOS 1, R2=dV LOS 2, R3=dV LOS 3</t>
+  </si>
+  <si>
+    <t>R1=d ang, R2=d alt, Search option</t>
+  </si>
+  <si>
+    <t>R1=dH (CDH), R2=dT, R3=dT</t>
+  </si>
+  <si>
+    <t>dVX,Y,Z (lcl vert)</t>
+  </si>
+  <si>
+    <t>dVX,Y,Z (LV) CDH</t>
+  </si>
+  <si>
+    <t>dVX,Y,Z (Body Control Axis)</t>
+  </si>
+  <si>
+    <t>dVX,Y,Z (Other Vehicle)</t>
+  </si>
+  <si>
+    <t>External dV</t>
+  </si>
+  <si>
+    <t>Target dV</t>
   </si>
 </sst>
 </file>
@@ -1640,10 +1640,10 @@
         <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" t="s">
         <v>230</v>
-      </c>
-      <c r="C1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1651,7 +1651,7 @@
         <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1659,7 +1659,7 @@
         <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1667,7 +1667,7 @@
         <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1675,7 +1675,7 @@
         <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1683,7 +1683,7 @@
         <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1691,7 +1691,7 @@
         <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>357</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1699,7 +1699,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1707,7 +1707,7 @@
         <v>71</v>
       </c>
       <c r="C9" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1715,7 +1715,7 @@
         <v>72</v>
       </c>
       <c r="C10" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1723,7 +1723,7 @@
         <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1731,7 +1731,7 @@
         <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1739,7 +1739,7 @@
         <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1747,7 +1747,7 @@
         <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1755,7 +1755,7 @@
         <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -1763,7 +1763,7 @@
         <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1771,7 +1771,7 @@
         <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -1779,7 +1779,7 @@
         <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -1787,7 +1787,7 @@
         <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1795,7 +1795,7 @@
         <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -2095,7 +2095,7 @@
         <v>115</v>
       </c>
       <c r="C53" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -2155,7 +2155,7 @@
         <v>121</v>
       </c>
       <c r="C59" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -2433,13 +2433,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" t="s">
         <v>232</v>
       </c>
-      <c r="B1" t="s">
-        <v>233</v>
-      </c>
       <c r="C1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -2447,7 +2447,7 @@
         <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="C2" t="s">
         <v>174</v>
@@ -2458,7 +2458,7 @@
         <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2466,7 +2466,7 @@
         <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="C4" t="s">
         <v>148</v>
@@ -2507,7 +2507,7 @@
         <v>167</v>
       </c>
       <c r="B8" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C8" t="s">
         <v>150</v>
@@ -2543,7 +2543,7 @@
         <v>154</v>
       </c>
       <c r="C11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -2565,7 +2565,7 @@
         <v>156</v>
       </c>
       <c r="C13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -2587,7 +2587,7 @@
         <v>157</v>
       </c>
       <c r="C15" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -2653,7 +2653,7 @@
         <v>165</v>
       </c>
       <c r="C21" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -2669,7 +2669,7 @@
         <v>172</v>
       </c>
       <c r="B23" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C23" t="s">
         <v>150</v>
@@ -2710,7 +2710,7 @@
         <v>182</v>
       </c>
       <c r="C27" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -2721,7 +2721,7 @@
         <v>183</v>
       </c>
       <c r="C28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -2732,7 +2732,7 @@
         <v>184</v>
       </c>
       <c r="C29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -2743,7 +2743,7 @@
         <v>185</v>
       </c>
       <c r="C30" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -2754,7 +2754,7 @@
         <v>186</v>
       </c>
       <c r="C31" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -2765,7 +2765,7 @@
         <v>187</v>
       </c>
       <c r="C32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -2776,7 +2776,7 @@
         <v>189</v>
       </c>
       <c r="C33" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -2784,10 +2784,10 @@
         <v>190</v>
       </c>
       <c r="B34" t="s">
-        <v>191</v>
+        <v>372</v>
       </c>
       <c r="C34" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -2795,10 +2795,10 @@
         <v>92</v>
       </c>
       <c r="B35" t="s">
-        <v>298</v>
+        <v>373</v>
       </c>
       <c r="C35" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -2806,10 +2806,10 @@
         <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C36" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -2817,10 +2817,10 @@
         <v>94</v>
       </c>
       <c r="B37" t="s">
-        <v>300</v>
+        <v>374</v>
       </c>
       <c r="C37" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -2828,10 +2828,10 @@
         <v>95</v>
       </c>
       <c r="B38" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="C38" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -2839,10 +2839,10 @@
         <v>96</v>
       </c>
       <c r="B39" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="C39" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -2850,10 +2850,10 @@
         <v>97</v>
       </c>
       <c r="B40" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C40" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -2861,7 +2861,7 @@
         <v>98</v>
       </c>
       <c r="B41" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C41" t="s">
         <v>150</v>
@@ -2872,10 +2872,10 @@
         <v>99</v>
       </c>
       <c r="B42" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C42" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -2883,10 +2883,10 @@
         <v>100</v>
       </c>
       <c r="B43" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -2894,10 +2894,10 @@
         <v>101</v>
       </c>
       <c r="B44" t="s">
-        <v>304</v>
+        <v>375</v>
       </c>
       <c r="C44" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -2905,10 +2905,10 @@
         <v>102</v>
       </c>
       <c r="B45" t="s">
-        <v>347</v>
+        <v>376</v>
       </c>
       <c r="C45" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -2916,7 +2916,7 @@
         <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C46" t="s">
         <v>148</v>
@@ -2927,7 +2927,7 @@
         <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C47" t="s">
         <v>148</v>
@@ -2938,10 +2938,10 @@
         <v>105</v>
       </c>
       <c r="B48" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C48" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -2949,10 +2949,10 @@
         <v>106</v>
       </c>
       <c r="B49" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C49" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -2960,10 +2960,10 @@
         <v>107</v>
       </c>
       <c r="B50" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C50" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -2971,10 +2971,10 @@
         <v>109</v>
       </c>
       <c r="B51" t="s">
-        <v>348</v>
+        <v>377</v>
       </c>
       <c r="C51" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -2982,10 +2982,10 @@
         <v>110</v>
       </c>
       <c r="B52" t="s">
-        <v>349</v>
+        <v>378</v>
       </c>
       <c r="C52" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -2993,10 +2993,10 @@
         <v>111</v>
       </c>
       <c r="B53" t="s">
-        <v>350</v>
+        <v>379</v>
       </c>
       <c r="C53" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -3004,10 +3004,10 @@
         <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="C54" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -3015,10 +3015,10 @@
         <v>113</v>
       </c>
       <c r="B55" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C55" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -3026,10 +3026,10 @@
         <v>114</v>
       </c>
       <c r="B56" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C56" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -3037,10 +3037,10 @@
         <v>115</v>
       </c>
       <c r="B57" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="C57" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -3048,10 +3048,10 @@
         <v>116</v>
       </c>
       <c r="B58" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="C58" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -3059,10 +3059,10 @@
         <v>117</v>
       </c>
       <c r="B59" t="s">
+        <v>215</v>
+      </c>
+      <c r="C59" t="s">
         <v>216</v>
-      </c>
-      <c r="C59" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -3070,10 +3070,10 @@
         <v>118</v>
       </c>
       <c r="B60" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="C60" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -3081,10 +3081,10 @@
         <v>119</v>
       </c>
       <c r="B61" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="C61" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -3092,10 +3092,10 @@
         <v>120</v>
       </c>
       <c r="B62" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="C62" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -3103,10 +3103,10 @@
         <v>121</v>
       </c>
       <c r="B63" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="C63" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -3114,7 +3114,7 @@
         <v>122</v>
       </c>
       <c r="B64" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C64" t="s">
         <v>150</v>
@@ -3125,7 +3125,7 @@
         <v>123</v>
       </c>
       <c r="B65" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C65" t="s">
         <v>150</v>
@@ -3136,10 +3136,10 @@
         <v>124</v>
       </c>
       <c r="B66" t="s">
-        <v>351</v>
+        <v>380</v>
       </c>
       <c r="C66" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -3147,10 +3147,10 @@
         <v>125</v>
       </c>
       <c r="B67" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="C67" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -3158,10 +3158,10 @@
         <v>126</v>
       </c>
       <c r="B68" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -3169,10 +3169,10 @@
         <v>127</v>
       </c>
       <c r="B69" t="s">
-        <v>352</v>
+        <v>381</v>
       </c>
       <c r="C69" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
@@ -3180,10 +3180,10 @@
         <v>131</v>
       </c>
       <c r="B70" t="s">
-        <v>298</v>
+        <v>373</v>
       </c>
       <c r="C70" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -3191,10 +3191,10 @@
         <v>132</v>
       </c>
       <c r="B71" t="s">
-        <v>353</v>
+        <v>382</v>
       </c>
       <c r="C71" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -3202,10 +3202,10 @@
         <v>133</v>
       </c>
       <c r="B72" t="s">
-        <v>354</v>
+        <v>383</v>
       </c>
       <c r="C72" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -3213,21 +3213,21 @@
         <v>134</v>
       </c>
       <c r="B73" t="s">
-        <v>355</v>
+        <v>384</v>
       </c>
       <c r="C73" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B74" t="s">
-        <v>356</v>
+        <v>385</v>
       </c>
       <c r="C74" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
@@ -3235,10 +3235,10 @@
         <v>135</v>
       </c>
       <c r="B75" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C75" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
@@ -3246,10 +3246,10 @@
         <v>137</v>
       </c>
       <c r="B76" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C76" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
@@ -3257,7 +3257,7 @@
         <v>138</v>
       </c>
       <c r="B77" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C77" t="s">
         <v>174</v>
@@ -3268,10 +3268,10 @@
         <v>139</v>
       </c>
       <c r="B78" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="C78" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -3279,10 +3279,10 @@
         <v>140</v>
       </c>
       <c r="B79" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="C79" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -3290,10 +3290,10 @@
         <v>141</v>
       </c>
       <c r="B80" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C80" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -3301,10 +3301,10 @@
         <v>142</v>
       </c>
       <c r="B81" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C81" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -3312,10 +3312,10 @@
         <v>143</v>
       </c>
       <c r="B82" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C82" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -3323,18 +3323,18 @@
         <v>144</v>
       </c>
       <c r="B83" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="C83" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B84" t="s">
         <v>237</v>
-      </c>
-      <c r="B84" t="s">
-        <v>238</v>
       </c>
       <c r="C84" t="s">
         <v>148</v>
@@ -3345,7 +3345,7 @@
         <v>145</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C85" t="s">
         <v>148</v>
@@ -3356,21 +3356,21 @@
         <v>146</v>
       </c>
       <c r="B86" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C86" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B87" t="s">
         <v>240</v>
       </c>
-      <c r="B87" t="s">
-        <v>241</v>
-      </c>
       <c r="C87" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
@@ -3378,10 +3378,10 @@
         <v>147</v>
       </c>
       <c r="B88" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C88" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -3402,18 +3402,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B1" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B2" t="s">
         <v>251</v>
-      </c>
-      <c r="B2" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -3421,7 +3421,7 @@
         <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -3429,7 +3429,7 @@
         <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -3437,7 +3437,7 @@
         <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -3445,7 +3445,7 @@
         <v>168</v>
       </c>
       <c r="B6" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -3453,7 +3453,7 @@
         <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -3461,7 +3461,7 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -3469,7 +3469,7 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -3477,7 +3477,7 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -3485,7 +3485,7 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -3493,15 +3493,15 @@
         <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B13" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -3509,7 +3509,7 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>259</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -3517,7 +3517,7 @@
         <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -3525,7 +3525,7 @@
         <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -3533,7 +3533,7 @@
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -3541,7 +3541,7 @@
         <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -3549,7 +3549,7 @@
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -3557,7 +3557,7 @@
         <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -3565,7 +3565,7 @@
         <v>188</v>
       </c>
       <c r="B21" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -3573,7 +3573,7 @@
         <v>190</v>
       </c>
       <c r="B22" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -3581,7 +3581,7 @@
         <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -3589,7 +3589,7 @@
         <v>41</v>
       </c>
       <c r="B24" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -3597,7 +3597,7 @@
         <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -3605,7 +3605,7 @@
         <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -3613,7 +3613,7 @@
         <v>52</v>
       </c>
       <c r="B27" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -3621,7 +3621,7 @@
         <v>105</v>
       </c>
       <c r="B28" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -3629,7 +3629,7 @@
         <v>106</v>
       </c>
       <c r="B29" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -3637,7 +3637,7 @@
         <v>61</v>
       </c>
       <c r="B30" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
@@ -3645,7 +3645,7 @@
         <v>114</v>
       </c>
       <c r="B31" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -3653,7 +3653,7 @@
         <v>115</v>
       </c>
       <c r="B32" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
@@ -3661,7 +3661,7 @@
         <v>116</v>
       </c>
       <c r="B33" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
@@ -3669,7 +3669,7 @@
         <v>117</v>
       </c>
       <c r="B34" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
@@ -3677,7 +3677,7 @@
         <v>118</v>
       </c>
       <c r="B35" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
@@ -3685,7 +3685,7 @@
         <v>119</v>
       </c>
       <c r="B36" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
@@ -3693,7 +3693,7 @@
         <v>124</v>
       </c>
       <c r="B37" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
@@ -3701,7 +3701,7 @@
         <v>125</v>
       </c>
       <c r="B38" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
@@ -3709,7 +3709,7 @@
         <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>271</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -3732,19 +3732,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="C1" t="s">
-        <v>364</v>
+        <v>348</v>
       </c>
       <c r="D1" t="s">
-        <v>365</v>
+        <v>349</v>
       </c>
       <c r="E1" t="s">
-        <v>366</v>
+        <v>350</v>
       </c>
       <c r="F1" t="s">
-        <v>367</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -3752,19 +3752,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>362</v>
+        <v>346</v>
       </c>
       <c r="C2" t="s">
-        <v>368</v>
+        <v>352</v>
       </c>
       <c r="D2" t="s">
-        <v>369</v>
+        <v>353</v>
       </c>
       <c r="E2" t="s">
-        <v>372</v>
+        <v>356</v>
       </c>
       <c r="F2" t="s">
-        <v>373</v>
+        <v>357</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3772,19 +3772,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C3" t="s">
+        <v>345</v>
+      </c>
+      <c r="D3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F3" t="s">
         <v>358</v>
-      </c>
-      <c r="C3" t="s">
-        <v>361</v>
-      </c>
-      <c r="D3" t="s">
-        <v>370</v>
-      </c>
-      <c r="E3" t="s">
-        <v>371</v>
-      </c>
-      <c r="F3" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3792,10 +3792,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>343</v>
+      </c>
+      <c r="F4" t="s">
         <v>359</v>
-      </c>
-      <c r="F4" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3803,10 +3803,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>344</v>
+      </c>
+      <c r="F5" t="s">
         <v>360</v>
-      </c>
-      <c r="F5" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3814,7 +3814,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>387</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -3835,19 +3835,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="C1" t="s">
-        <v>364</v>
+        <v>348</v>
       </c>
       <c r="D1" t="s">
-        <v>365</v>
+        <v>349</v>
       </c>
       <c r="E1" t="s">
-        <v>366</v>
+        <v>350</v>
       </c>
       <c r="F1" t="s">
-        <v>367</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -3855,19 +3855,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>377</v>
+        <v>361</v>
       </c>
       <c r="C2" t="s">
-        <v>385</v>
+        <v>369</v>
       </c>
       <c r="D2" t="s">
-        <v>384</v>
+        <v>368</v>
       </c>
       <c r="E2" t="s">
-        <v>380</v>
+        <v>364</v>
       </c>
       <c r="F2" t="s">
-        <v>382</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3875,19 +3875,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>386</v>
+        <v>370</v>
       </c>
       <c r="C3" t="s">
-        <v>378</v>
+        <v>362</v>
       </c>
       <c r="D3" t="s">
-        <v>379</v>
+        <v>363</v>
       </c>
       <c r="E3" t="s">
-        <v>381</v>
+        <v>365</v>
       </c>
       <c r="F3" t="s">
-        <v>383</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
found the degrees symbol does not work sometimes, replaced with deg instead
</commit_message>
<xml_diff>
--- a/CSM/CSM Verb and noun list.xlsx
+++ b/CSM/CSM Verb and noun list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\del13\nassp-checklist-annotator\CSM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A06BFA-0BBE-4C49-91F3-04D871F50276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F103B31-4E3A-488F-90F6-0AEDDB8C76AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20676" windowHeight="16560" activeTab="1" xr2:uid="{424832EF-970A-4448-8501-E17666F9A823}"/>
+    <workbookView xWindow="20388" yWindow="0" windowWidth="20664" windowHeight="16560" activeTab="3" xr2:uid="{424832EF-970A-4448-8501-E17666F9A823}"/>
   </bookViews>
   <sheets>
     <sheet name="Verb" sheetId="1" r:id="rId1"/>
@@ -523,9 +523,6 @@
     <t>99</t>
   </si>
   <si>
-    <t>.01°</t>
-  </si>
-  <si>
     <t>Angular Error/Diff</t>
   </si>
   <si>
@@ -556,9 +553,6 @@
     <t>Astronaut total att</t>
   </si>
   <si>
-    <t>R,P,Y .01°</t>
-  </si>
-  <si>
     <t>Auto Maneuver</t>
   </si>
   <si>
@@ -658,18 +652,12 @@
     <t>.1 NM .1 NM .1 FPS</t>
   </si>
   <si>
-    <t>XXBXX min-sec .01°</t>
-  </si>
-  <si>
     <t>DAP Config (R1&amp;R2)</t>
   </si>
   <si>
     <t>LBS LBS</t>
   </si>
   <si>
-    <t>.01° .01°</t>
-  </si>
-  <si>
     <t>.1 NM .1 FPS 0000X.</t>
   </si>
   <si>
@@ -691,21 +679,9 @@
     <t>.1 NM .1 NM min-sec</t>
   </si>
   <si>
-    <t>.01 NM .1 FPS .01°</t>
-  </si>
-  <si>
-    <t>CODE .01° .01°</t>
-  </si>
-  <si>
     <t>.1 NM .1 FPS .1 FPS</t>
   </si>
   <si>
-    <t>.01 G FPS .01°</t>
-  </si>
-  <si>
-    <t>.01° .01° +/-00001</t>
-  </si>
-  <si>
     <t>FPS FPS .1 NM</t>
   </si>
   <si>
@@ -721,48 +697,18 @@
     <t>VGX,Y,Z (Body Control Axis)</t>
   </si>
   <si>
-    <t>.001°</t>
-  </si>
-  <si>
     <t>Sampled CMC Time (fetched in interrupt)</t>
   </si>
   <si>
     <t>hrs min .01 sec</t>
   </si>
   <si>
-    <t>.01° .1 NM .1 NM</t>
-  </si>
-  <si>
-    <t>.1 NM .01° .01°</t>
-  </si>
-  <si>
-    <t>.01° FPS FPS</t>
-  </si>
-  <si>
-    <t>.01° .01 G FPS</t>
-  </si>
-  <si>
-    <t>.01° .1 NM</t>
-  </si>
-  <si>
-    <t>10 NM FPS .01°</t>
-  </si>
-  <si>
-    <t>.01° .001° 0000X</t>
-  </si>
-  <si>
-    <t>.01° FPS .01 G</t>
-  </si>
-  <si>
     <t>.1 NM min-sec min-sec</t>
   </si>
   <si>
     <t>min-sec FPS FPS</t>
   </si>
   <si>
-    <t>.01° .001°</t>
-  </si>
-  <si>
     <t>Opt Calib Data - Shaft (R1), Trunnion(R2)</t>
   </si>
   <si>
@@ -805,9 +751,6 @@
     <t>Planet X Y Z</t>
   </si>
   <si>
-    <t>.001° .001° .01 NM</t>
-  </si>
-  <si>
     <t>+X axis att ICDU angles</t>
   </si>
   <si>
@@ -823,9 +766,6 @@
     <t>Noun Scale</t>
   </si>
   <si>
-    <t>.01° .01° .1 NM</t>
-  </si>
-  <si>
     <t>Monitor Decimal</t>
   </si>
   <si>
@@ -1144,24 +1084,6 @@
     <t>B/D=1=Use</t>
   </si>
   <si>
-    <t>DB=1=5.0°</t>
-  </si>
-  <si>
-    <t>DB=0=0.5°</t>
-  </si>
-  <si>
-    <t>RATE=0=0.05°/sec</t>
-  </si>
-  <si>
-    <t>RATE=1=0.2°/sec</t>
-  </si>
-  <si>
-    <t>RATE=2=0.5°/sec</t>
-  </si>
-  <si>
-    <t>RATE=3=2.0°/sec</t>
-  </si>
-  <si>
     <t>ROLLQD=0=B/D</t>
   </si>
   <si>
@@ -1241,6 +1163,84 @@
   </si>
   <si>
     <t>Target dV</t>
+  </si>
+  <si>
+    <t>.01deg</t>
+  </si>
+  <si>
+    <t>R,P,Y .01deg</t>
+  </si>
+  <si>
+    <t>.01deg .001deg 0000X</t>
+  </si>
+  <si>
+    <t>.01deg .01deg .1 NM</t>
+  </si>
+  <si>
+    <t>XXBXX min-sec .01deg</t>
+  </si>
+  <si>
+    <t>.01deg .01deg</t>
+  </si>
+  <si>
+    <t>.01 NM .1 FPS .01deg</t>
+  </si>
+  <si>
+    <t>CODE .01deg .01deg</t>
+  </si>
+  <si>
+    <t>.01 G FPS .01deg</t>
+  </si>
+  <si>
+    <t>.01deg .01deg +/-00001</t>
+  </si>
+  <si>
+    <t>.01deg .1 NM .1 NM</t>
+  </si>
+  <si>
+    <t>.1 NM .01deg .01deg</t>
+  </si>
+  <si>
+    <t>.01deg FPS FPS</t>
+  </si>
+  <si>
+    <t>.01deg .01 G FPS</t>
+  </si>
+  <si>
+    <t>.01deg .1 NM</t>
+  </si>
+  <si>
+    <t>10 NM FPS .01deg</t>
+  </si>
+  <si>
+    <t>.01deg FPS .01 G</t>
+  </si>
+  <si>
+    <t>.01deg .001deg</t>
+  </si>
+  <si>
+    <t>.001deg .001deg .01 NM</t>
+  </si>
+  <si>
+    <t>.001deg</t>
+  </si>
+  <si>
+    <t>DB=0=0.5deg</t>
+  </si>
+  <si>
+    <t>RATE=0=0.05deg/sec</t>
+  </si>
+  <si>
+    <t>DB=1=5.0deg</t>
+  </si>
+  <si>
+    <t>RATE=1=0.2deg/sec</t>
+  </si>
+  <si>
+    <t>RATE=2=0.5deg/sec</t>
+  </si>
+  <si>
+    <t>RATE=3=2.0deg/sec</t>
   </si>
 </sst>
 </file>
@@ -1640,10 +1640,10 @@
         <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="C1" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1651,7 +1651,7 @@
         <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>322</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1659,7 +1659,7 @@
         <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>323</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1667,7 +1667,7 @@
         <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>324</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1675,7 +1675,7 @@
         <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1683,7 +1683,7 @@
         <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>326</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1691,7 +1691,7 @@
         <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>341</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1699,7 +1699,7 @@
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>327</v>
+        <v>307</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1707,7 +1707,7 @@
         <v>71</v>
       </c>
       <c r="C9" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1715,7 +1715,7 @@
         <v>72</v>
       </c>
       <c r="C10" t="s">
-        <v>329</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1723,7 +1723,7 @@
         <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1731,7 +1731,7 @@
         <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>331</v>
+        <v>311</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1739,7 +1739,7 @@
         <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1747,7 +1747,7 @@
         <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1755,7 +1755,7 @@
         <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -1763,7 +1763,7 @@
         <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>334</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1771,7 +1771,7 @@
         <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>335</v>
+        <v>315</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -1779,7 +1779,7 @@
         <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>336</v>
+        <v>316</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -1787,7 +1787,7 @@
         <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>337</v>
+        <v>317</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1795,7 +1795,7 @@
         <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>338</v>
+        <v>318</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -2095,7 +2095,7 @@
         <v>115</v>
       </c>
       <c r="C53" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -2155,7 +2155,7 @@
         <v>121</v>
       </c>
       <c r="C59" t="s">
-        <v>321</v>
+        <v>301</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -2389,7 +2389,7 @@
         <v>145</v>
       </c>
       <c r="C83" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
@@ -2410,7 +2410,7 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2433,13 +2433,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
       <c r="B1" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="C1" t="s">
-        <v>247</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -2447,10 +2447,10 @@
         <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
       <c r="C2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -2458,7 +2458,7 @@
         <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2466,10 +2466,10 @@
         <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -2477,10 +2477,10 @@
         <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C5" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2488,10 +2488,10 @@
         <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2499,40 +2499,40 @@
         <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B8" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="C8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -2540,10 +2540,10 @@
         <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -2551,10 +2551,10 @@
         <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -2562,10 +2562,10 @@
         <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C13" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -2573,10 +2573,10 @@
         <v>75</v>
       </c>
       <c r="B14" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -2584,10 +2584,10 @@
         <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C15" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -2595,32 +2595,32 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C16" t="s">
-        <v>159</v>
+        <v>363</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B17" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C17" t="s">
-        <v>159</v>
+        <v>363</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B18" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C18" t="s">
-        <v>159</v>
+        <v>363</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -2628,10 +2628,10 @@
         <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -2639,10 +2639,10 @@
         <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C20" t="s">
-        <v>159</v>
+        <v>363</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -2650,10 +2650,10 @@
         <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -2661,18 +2661,18 @@
         <v>82</v>
       </c>
       <c r="B22" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B23" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="C23" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -2680,18 +2680,18 @@
         <v>83</v>
       </c>
       <c r="B24" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C25" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -2699,7 +2699,7 @@
         <v>84</v>
       </c>
       <c r="B26" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -2707,10 +2707,10 @@
         <v>86</v>
       </c>
       <c r="B27" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C27" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -2718,10 +2718,10 @@
         <v>87</v>
       </c>
       <c r="B28" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C28" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -2729,10 +2729,10 @@
         <v>88</v>
       </c>
       <c r="B29" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C29" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -2740,10 +2740,10 @@
         <v>89</v>
       </c>
       <c r="B30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C30" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -2751,10 +2751,10 @@
         <v>90</v>
       </c>
       <c r="B31" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C31" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -2762,32 +2762,32 @@
         <v>91</v>
       </c>
       <c r="B32" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C32" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B33" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C33" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B34" t="s">
-        <v>372</v>
+        <v>346</v>
       </c>
       <c r="C34" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -2795,10 +2795,10 @@
         <v>92</v>
       </c>
       <c r="B35" t="s">
-        <v>373</v>
+        <v>347</v>
       </c>
       <c r="C35" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -2806,10 +2806,10 @@
         <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="C36" t="s">
-        <v>223</v>
+        <v>364</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -2817,10 +2817,10 @@
         <v>94</v>
       </c>
       <c r="B37" t="s">
-        <v>374</v>
+        <v>348</v>
       </c>
       <c r="C37" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -2828,10 +2828,10 @@
         <v>95</v>
       </c>
       <c r="B38" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="C38" t="s">
-        <v>248</v>
+        <v>365</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -2839,10 +2839,10 @@
         <v>96</v>
       </c>
       <c r="B39" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="C39" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -2850,10 +2850,10 @@
         <v>97</v>
       </c>
       <c r="B40" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="C40" t="s">
-        <v>193</v>
+        <v>366</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -2861,10 +2861,10 @@
         <v>98</v>
       </c>
       <c r="B41" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C41" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -2872,10 +2872,10 @@
         <v>99</v>
       </c>
       <c r="B42" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
       <c r="C42" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -2883,10 +2883,10 @@
         <v>100</v>
       </c>
       <c r="B43" t="s">
-        <v>292</v>
+        <v>272</v>
       </c>
       <c r="C43" t="s">
-        <v>196</v>
+        <v>367</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -2894,10 +2894,10 @@
         <v>101</v>
       </c>
       <c r="B44" t="s">
-        <v>375</v>
+        <v>349</v>
       </c>
       <c r="C44" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -2905,10 +2905,10 @@
         <v>102</v>
       </c>
       <c r="B45" t="s">
-        <v>376</v>
+        <v>350</v>
       </c>
       <c r="C45" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -2916,10 +2916,10 @@
         <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>293</v>
+        <v>273</v>
       </c>
       <c r="C46" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -2927,10 +2927,10 @@
         <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C47" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -2938,10 +2938,10 @@
         <v>105</v>
       </c>
       <c r="B48" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="C48" t="s">
-        <v>204</v>
+        <v>368</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -2949,10 +2949,10 @@
         <v>106</v>
       </c>
       <c r="B49" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="C49" t="s">
-        <v>204</v>
+        <v>368</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -2960,10 +2960,10 @@
         <v>107</v>
       </c>
       <c r="B50" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
       <c r="C50" t="s">
-        <v>205</v>
+        <v>369</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -2971,10 +2971,10 @@
         <v>109</v>
       </c>
       <c r="B51" t="s">
-        <v>377</v>
+        <v>351</v>
       </c>
       <c r="C51" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -2982,10 +2982,10 @@
         <v>110</v>
       </c>
       <c r="B52" t="s">
-        <v>378</v>
+        <v>352</v>
       </c>
       <c r="C52" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -2993,10 +2993,10 @@
         <v>111</v>
       </c>
       <c r="B53" t="s">
-        <v>379</v>
+        <v>353</v>
       </c>
       <c r="C53" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -3004,10 +3004,10 @@
         <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="C54" t="s">
-        <v>207</v>
+        <v>370</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -3015,10 +3015,10 @@
         <v>113</v>
       </c>
       <c r="B55" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="C55" t="s">
-        <v>208</v>
+        <v>371</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -3026,10 +3026,10 @@
         <v>114</v>
       </c>
       <c r="B56" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="C56" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -3037,10 +3037,10 @@
         <v>115</v>
       </c>
       <c r="B57" t="s">
-        <v>305</v>
+        <v>285</v>
       </c>
       <c r="C57" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -3048,10 +3048,10 @@
         <v>116</v>
       </c>
       <c r="B58" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
       <c r="C58" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -3059,10 +3059,10 @@
         <v>117</v>
       </c>
       <c r="B59" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="C59" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -3070,10 +3070,10 @@
         <v>118</v>
       </c>
       <c r="B60" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="C60" t="s">
-        <v>217</v>
+        <v>372</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -3081,10 +3081,10 @@
         <v>119</v>
       </c>
       <c r="B61" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="C61" t="s">
-        <v>218</v>
+        <v>373</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -3092,10 +3092,10 @@
         <v>120</v>
       </c>
       <c r="B62" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="C62" t="s">
-        <v>219</v>
+        <v>374</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -3103,10 +3103,10 @@
         <v>121</v>
       </c>
       <c r="B63" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="C63" t="s">
-        <v>220</v>
+        <v>375</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -3114,10 +3114,10 @@
         <v>122</v>
       </c>
       <c r="B64" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
       <c r="C64" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
@@ -3125,10 +3125,10 @@
         <v>123</v>
       </c>
       <c r="B65" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="C65" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
@@ -3136,10 +3136,10 @@
         <v>124</v>
       </c>
       <c r="B66" t="s">
-        <v>380</v>
+        <v>354</v>
       </c>
       <c r="C66" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -3147,10 +3147,10 @@
         <v>125</v>
       </c>
       <c r="B67" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="C67" t="s">
-        <v>222</v>
+        <v>377</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -3158,10 +3158,10 @@
         <v>126</v>
       </c>
       <c r="B68" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="C68" t="s">
-        <v>224</v>
+        <v>378</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -3169,10 +3169,10 @@
         <v>127</v>
       </c>
       <c r="B69" t="s">
-        <v>381</v>
+        <v>355</v>
       </c>
       <c r="C69" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
@@ -3180,10 +3180,10 @@
         <v>131</v>
       </c>
       <c r="B70" t="s">
-        <v>373</v>
+        <v>347</v>
       </c>
       <c r="C70" t="s">
-        <v>226</v>
+        <v>209</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -3191,10 +3191,10 @@
         <v>132</v>
       </c>
       <c r="B71" t="s">
-        <v>382</v>
+        <v>356</v>
       </c>
       <c r="C71" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -3202,10 +3202,10 @@
         <v>133</v>
       </c>
       <c r="B72" t="s">
-        <v>383</v>
+        <v>357</v>
       </c>
       <c r="C72" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -3213,21 +3213,21 @@
         <v>134</v>
       </c>
       <c r="B73" t="s">
-        <v>384</v>
+        <v>358</v>
       </c>
       <c r="C73" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="B74" t="s">
-        <v>385</v>
+        <v>359</v>
       </c>
       <c r="C74" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
@@ -3235,10 +3235,10 @@
         <v>135</v>
       </c>
       <c r="B75" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C75" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
@@ -3246,10 +3246,10 @@
         <v>137</v>
       </c>
       <c r="B76" t="s">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="C76" t="s">
-        <v>227</v>
+        <v>379</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
@@ -3257,10 +3257,10 @@
         <v>138</v>
       </c>
       <c r="B77" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="C77" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -3268,10 +3268,10 @@
         <v>139</v>
       </c>
       <c r="B78" t="s">
-        <v>340</v>
+        <v>320</v>
       </c>
       <c r="C78" t="s">
-        <v>242</v>
+        <v>380</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -3279,10 +3279,10 @@
         <v>140</v>
       </c>
       <c r="B79" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="C79" t="s">
-        <v>204</v>
+        <v>368</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -3290,10 +3290,10 @@
         <v>141</v>
       </c>
       <c r="B80" t="s">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="C80" t="s">
-        <v>227</v>
+        <v>379</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -3301,10 +3301,10 @@
         <v>142</v>
       </c>
       <c r="B81" t="s">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="C81" t="s">
-        <v>227</v>
+        <v>379</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -3312,10 +3312,10 @@
         <v>143</v>
       </c>
       <c r="B82" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="C82" t="s">
-        <v>214</v>
+        <v>381</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -3323,21 +3323,21 @@
         <v>144</v>
       </c>
       <c r="B83" t="s">
-        <v>339</v>
+        <v>319</v>
       </c>
       <c r="C83" t="s">
-        <v>227</v>
+        <v>379</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
-        <v>236</v>
+        <v>218</v>
       </c>
       <c r="B84" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="C84" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
@@ -3345,10 +3345,10 @@
         <v>145</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>243</v>
+        <v>224</v>
       </c>
       <c r="C85" t="s">
-        <v>148</v>
+        <v>362</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -3356,21 +3356,21 @@
         <v>146</v>
       </c>
       <c r="B86" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="C86" t="s">
-        <v>245</v>
+        <v>226</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="B87" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="C87" t="s">
-        <v>246</v>
+        <v>227</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
@@ -3378,10 +3378,10 @@
         <v>147</v>
       </c>
       <c r="B88" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
       <c r="C88" t="s">
-        <v>244</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -3402,18 +3402,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="B1" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -3421,7 +3421,7 @@
         <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -3429,7 +3429,7 @@
         <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -3437,15 +3437,15 @@
         <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B6" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -3453,7 +3453,7 @@
         <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -3461,7 +3461,7 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -3469,7 +3469,7 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -3477,7 +3477,7 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -3485,7 +3485,7 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -3493,15 +3493,15 @@
         <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="B13" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -3509,7 +3509,7 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>386</v>
+        <v>360</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -3517,7 +3517,7 @@
         <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -3525,7 +3525,7 @@
         <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -3533,7 +3533,7 @@
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -3541,7 +3541,7 @@
         <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -3549,7 +3549,7 @@
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -3557,23 +3557,23 @@
         <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B21" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B22" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -3581,7 +3581,7 @@
         <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -3589,7 +3589,7 @@
         <v>41</v>
       </c>
       <c r="B24" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -3597,7 +3597,7 @@
         <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -3605,7 +3605,7 @@
         <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -3613,7 +3613,7 @@
         <v>52</v>
       </c>
       <c r="B27" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -3621,7 +3621,7 @@
         <v>105</v>
       </c>
       <c r="B28" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -3629,7 +3629,7 @@
         <v>106</v>
       </c>
       <c r="B29" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -3637,7 +3637,7 @@
         <v>61</v>
       </c>
       <c r="B30" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
@@ -3645,7 +3645,7 @@
         <v>114</v>
       </c>
       <c r="B31" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -3653,7 +3653,7 @@
         <v>115</v>
       </c>
       <c r="B32" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
@@ -3661,7 +3661,7 @@
         <v>116</v>
       </c>
       <c r="B33" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
@@ -3669,7 +3669,7 @@
         <v>117</v>
       </c>
       <c r="B34" t="s">
-        <v>288</v>
+        <v>268</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
@@ -3677,7 +3677,7 @@
         <v>118</v>
       </c>
       <c r="B35" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
@@ -3685,7 +3685,7 @@
         <v>119</v>
       </c>
       <c r="B36" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
@@ -3693,7 +3693,7 @@
         <v>124</v>
       </c>
       <c r="B37" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
@@ -3701,7 +3701,7 @@
         <v>125</v>
       </c>
       <c r="B38" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
@@ -3709,7 +3709,7 @@
         <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>387</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -3726,25 +3726,25 @@
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" customWidth="1"/>
     <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>347</v>
+        <v>327</v>
       </c>
       <c r="C1" t="s">
-        <v>348</v>
+        <v>328</v>
       </c>
       <c r="D1" t="s">
-        <v>349</v>
+        <v>329</v>
       </c>
       <c r="E1" t="s">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="F1" t="s">
-        <v>351</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -3752,19 +3752,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>346</v>
+        <v>326</v>
       </c>
       <c r="C2" t="s">
-        <v>352</v>
+        <v>332</v>
       </c>
       <c r="D2" t="s">
-        <v>353</v>
+        <v>333</v>
       </c>
       <c r="E2" t="s">
-        <v>356</v>
+        <v>382</v>
       </c>
       <c r="F2" t="s">
-        <v>357</v>
+        <v>383</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3772,19 +3772,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>342</v>
+        <v>322</v>
       </c>
       <c r="C3" t="s">
-        <v>345</v>
+        <v>325</v>
       </c>
       <c r="D3" t="s">
-        <v>354</v>
+        <v>334</v>
       </c>
       <c r="E3" t="s">
-        <v>355</v>
+        <v>384</v>
       </c>
       <c r="F3" t="s">
-        <v>358</v>
+        <v>385</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3792,10 +3792,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>343</v>
+        <v>323</v>
       </c>
       <c r="F4" t="s">
-        <v>359</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3803,10 +3803,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>344</v>
+        <v>324</v>
       </c>
       <c r="F5" t="s">
-        <v>360</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3814,7 +3814,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>371</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -3835,19 +3835,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>347</v>
+        <v>327</v>
       </c>
       <c r="C1" t="s">
-        <v>348</v>
+        <v>328</v>
       </c>
       <c r="D1" t="s">
-        <v>349</v>
+        <v>329</v>
       </c>
       <c r="E1" t="s">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="F1" t="s">
-        <v>351</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -3855,19 +3855,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>361</v>
+        <v>335</v>
       </c>
       <c r="C2" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="D2" t="s">
-        <v>368</v>
+        <v>342</v>
       </c>
       <c r="E2" t="s">
-        <v>364</v>
+        <v>338</v>
       </c>
       <c r="F2" t="s">
-        <v>366</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3875,19 +3875,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="C3" t="s">
-        <v>362</v>
+        <v>336</v>
       </c>
       <c r="D3" t="s">
-        <v>363</v>
+        <v>337</v>
       </c>
       <c r="E3" t="s">
-        <v>365</v>
+        <v>339</v>
       </c>
       <c r="F3" t="s">
-        <v>367</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>